<commit_message>
CTD data are ready for CMAP
</commit_message>
<xml_diff>
--- a/CMAP_variableMetadata_additions.xlsx
+++ b/CMAP_variableMetadata_additions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\GitHub_niskin\BWrepos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A936B9-851A-40C3-83FF-42F3B81EFDF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F91F649E-C51D-4054-A48D-EA0DE5F0D34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27255" yWindow="4380" windowWidth="23100" windowHeight="16170" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27630" yWindow="3885" windowWidth="26595" windowHeight="16365" firstSheet="4" activeTab="8" xr2:uid="{838CA6DE-4AAC-45DB-B6F8-47923BA10D1F}"/>
   </bookViews>
   <sheets>
     <sheet name="notes" sheetId="4" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="964684_v1_amino_acids_biosscope" sheetId="9" r:id="rId6"/>
     <sheet name="920443_v1_biosscope_in_situ_pum" sheetId="10" r:id="rId7"/>
     <sheet name="PVST_BATS_PLANKTON" sheetId="11" r:id="rId8"/>
-    <sheet name="all_temp" sheetId="12" r:id="rId9"/>
+    <sheet name="1000939_v1_bios_scope_ctd" sheetId="13" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">PVST_BATS_PLANKTON!$A$5:$I$73</definedName>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2579" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2325" uniqueCount="615">
   <si>
     <t>Program</t>
   </si>
@@ -1246,9 +1246,6 @@
     <t>hh:mm:ss</t>
   </si>
   <si>
-    <t>BIOS-SCOPE, BIOS, Simons Foundation International, bio, biogeo, biogeochemistry, biology, flowCAM, Zooscan, net tows, Discrete, Bottle, cruise, Discrete, in situ, insitu, in-situ, North Atlantic Ocean, observation</t>
-  </si>
-  <si>
     <t>degrees</t>
   </si>
   <si>
@@ -1558,9 +1555,6 @@
     <t>biovolume</t>
   </si>
   <si>
-    <t>Biovolume for the target detected within the ROI determined by means specified in the biovolume calculation method or protocol document.</t>
-  </si>
-  <si>
     <t>um^3</t>
   </si>
   <si>
@@ -1721,6 +1715,180 @@
   </si>
   <si>
     <t>use this to distinguish between different types of flowcam samples</t>
+  </si>
+  <si>
+    <t>cast</t>
+  </si>
+  <si>
+    <t>dimensionless</t>
+  </si>
+  <si>
+    <t>HHMM</t>
+  </si>
+  <si>
+    <t>decibars (db)</t>
+  </si>
+  <si>
+    <t>fluor</t>
+  </si>
+  <si>
+    <t>par</t>
+  </si>
+  <si>
+    <t>BIOS-SCOPE, BIOS, Simons Foundation International,  cruise, in situ, insitu, in-situ, North Atlantic Ocean, observation</t>
+  </si>
+  <si>
+    <t>Consecutive cast number for the instrument</t>
+  </si>
+  <si>
+    <t>par0</t>
+  </si>
+  <si>
+    <t>z_par_1pcnt</t>
+  </si>
+  <si>
+    <t>z_par_halfpcnt</t>
+  </si>
+  <si>
+    <t>z_par_tenthpcnt</t>
+  </si>
+  <si>
+    <t>pr</t>
+  </si>
+  <si>
+    <t>te</t>
+  </si>
+  <si>
+    <t>co</t>
+  </si>
+  <si>
+    <t>sa</t>
+  </si>
+  <si>
+    <t>o2</t>
+  </si>
+  <si>
+    <t>bac</t>
+  </si>
+  <si>
+    <t>fluor_filt</t>
+  </si>
+  <si>
+    <t>par_est</t>
+  </si>
+  <si>
+    <t>th</t>
+  </si>
+  <si>
+    <t>sig0</t>
+  </si>
+  <si>
+    <t>rho</t>
+  </si>
+  <si>
+    <t>bvfrq</t>
+  </si>
+  <si>
+    <t>vertZone</t>
+  </si>
+  <si>
+    <t>Cruise number</t>
+  </si>
+  <si>
+    <t>Mixed layer depth defined by surface density + 0.125 kg/m^3 (Suga, T., K. Motoki, Y. Aoki, and A. M. Macdonald (2004), The North Pacific climatology of winter mixed layer and mode waters, J. Phys. Oceanogr., 34, 3 – 22,10.1175/1520-0485(2004)034&lt;0003:TNPCOW&gt;2.0.CO;2)</t>
+  </si>
+  <si>
+    <t>Depth of 'active mixing' defined by buoyancy frequency (Morison, F., E. Harvey, G. Franzè and S. Menden-Deuer (2019). Storm-Induced Predator-Prey Decoupling Promotes Springtime Accumulation of North Atlantic Phytoplankton. Frontiers in Marine Science Volume 6 - 2019. DOI: 10.3389/fmars.2019.00608) and (Graff, J. R. and M. J. Behrenfeld (2018). Photoacclimation Responses in Subarctic Atlantic Phytoplankton Following a Natural Mixing-Restratification Event. Frontiers in Marine Science Volume 5 - 2018. DOI: 10.3389/fmars.2018.00209)"</t>
+  </si>
+  <si>
+    <t>meters</t>
+  </si>
+  <si>
+    <t>MLD from Thermal Expansion Coeff, and dT=0.2 deg C (Sprintall, J., and M. Tomczak (1992), Evidence of the barrier layer in the surface layer of the tropics, J. Geophys. Res., 97, 7305– 7316,10.1029/92JC00407)</t>
+  </si>
+  <si>
+    <t>Season designation (1 = mixed, 2  = spring, 3 = stratified, 4 = fall)</t>
+  </si>
+  <si>
+    <t>Surface PAR value</t>
+  </si>
+  <si>
+    <t>microeinsteins per meter squared per second (uE/m2/s)</t>
+  </si>
+  <si>
+    <t>Depth of 1% light level</t>
+  </si>
+  <si>
+    <t>Depth of 0.5% light level</t>
+  </si>
+  <si>
+    <t>Depth of 0.1% light level</t>
+  </si>
+  <si>
+    <t>time of sunrise</t>
+  </si>
+  <si>
+    <t>time of sunset</t>
+  </si>
+  <si>
+    <t>Vertical Zone designation (see description in Curry et al. 2026)</t>
+  </si>
+  <si>
+    <t>Brunt-Vaisala Frequency squared (N^2)</t>
+  </si>
+  <si>
+    <t>Density of seawater</t>
+  </si>
+  <si>
+    <t>Potential temperature as per UNESCO 1983 report</t>
+  </si>
+  <si>
+    <t>Photosynthetically Active Radiation (PAR): fitted exponential profile</t>
+  </si>
+  <si>
+    <t>Photosynthetically Active Radiation (PAR)</t>
+  </si>
+  <si>
+    <t>Fluorescence filtered (applies a 3rd order butterworth filter to the fluorometer profile)</t>
+  </si>
+  <si>
+    <t>Fluorescence</t>
+  </si>
+  <si>
+    <t>Beam Attenuation Coefficient</t>
+  </si>
+  <si>
+    <t>Dissolved Oxygen</t>
+  </si>
+  <si>
+    <t>PSU</t>
+  </si>
+  <si>
+    <t>Salinity</t>
+  </si>
+  <si>
+    <t>Temperature (ITS-90)</t>
+  </si>
+  <si>
+    <t>S/m</t>
+  </si>
+  <si>
+    <t>reciprocal meters (1/m)</t>
+  </si>
+  <si>
+    <t>relative fluorescence units (RFU)</t>
+  </si>
+  <si>
+    <t>degree C (ITS-90)</t>
+  </si>
+  <si>
+    <t>Potential density relative to the reference pressure</t>
+  </si>
+  <si>
+    <t>kg/m^3</t>
+  </si>
+  <si>
+    <t>s^-2</t>
   </si>
 </sst>
 </file>
@@ -7586,27 +7754,27 @@
         <v>150</v>
       </c>
       <c r="G2" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B3" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="C3" t="s">
         <v>387</v>
       </c>
       <c r="D3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E3" t="s">
         <v>150</v>
@@ -7615,27 +7783,27 @@
         <v>150</v>
       </c>
       <c r="G3" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>401</v>
+      </c>
+      <c r="B4" t="s">
         <v>402</v>
       </c>
-      <c r="B4" t="s">
-        <v>403</v>
-      </c>
       <c r="C4" t="s">
         <v>387</v>
       </c>
       <c r="D4" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E4" t="s">
         <v>150</v>
@@ -7644,21 +7812,21 @@
         <v>150</v>
       </c>
       <c r="G4" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
+        <v>403</v>
+      </c>
+      <c r="B5" t="s">
         <v>404</v>
-      </c>
-      <c r="B5" t="s">
-        <v>405</v>
       </c>
       <c r="C5" t="s">
         <v>387</v>
@@ -7673,27 +7841,27 @@
         <v>150</v>
       </c>
       <c r="G5" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="B6" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="C6" t="s">
         <v>387</v>
       </c>
       <c r="D6" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E6" t="s">
         <v>150</v>
@@ -7702,28 +7870,28 @@
         <v>150</v>
       </c>
       <c r="G6" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
+        <v>405</v>
+      </c>
+      <c r="B7" t="s">
         <v>406</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>387</v>
+      </c>
+      <c r="D7" t="s">
         <v>407</v>
       </c>
-      <c r="C7" t="s">
-        <v>387</v>
-      </c>
-      <c r="D7" t="s">
-        <v>408</v>
-      </c>
       <c r="E7" t="s">
         <v>150</v>
       </c>
@@ -7731,27 +7899,27 @@
         <v>150</v>
       </c>
       <c r="G7" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="I7" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
+        <v>408</v>
+      </c>
+      <c r="B8" t="s">
         <v>409</v>
       </c>
-      <c r="B8" t="s">
-        <v>410</v>
-      </c>
       <c r="C8" t="s">
         <v>387</v>
       </c>
       <c r="D8" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E8" t="s">
         <v>150</v>
@@ -7760,21 +7928,21 @@
         <v>150</v>
       </c>
       <c r="G8" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B9" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C9" t="s">
         <v>387</v>
@@ -7795,15 +7963,15 @@
         <v>0</v>
       </c>
       <c r="I9" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
+        <v>410</v>
+      </c>
+      <c r="B10" t="s">
         <v>411</v>
-      </c>
-      <c r="B10" t="s">
-        <v>412</v>
       </c>
       <c r="C10" t="s">
         <v>387</v>
@@ -7818,27 +7986,27 @@
         <v>150</v>
       </c>
       <c r="G10" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
+        <v>412</v>
+      </c>
+      <c r="B11" t="s">
         <v>413</v>
       </c>
-      <c r="B11" t="s">
-        <v>414</v>
-      </c>
       <c r="C11" t="s">
         <v>387</v>
       </c>
       <c r="D11" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E11" t="s">
         <v>150</v>
@@ -7847,28 +8015,28 @@
         <v>150</v>
       </c>
       <c r="G11" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
+        <v>414</v>
+      </c>
+      <c r="B12" t="s">
         <v>415</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>387</v>
+      </c>
+      <c r="D12" t="s">
         <v>416</v>
       </c>
-      <c r="C12" t="s">
-        <v>387</v>
-      </c>
-      <c r="D12" t="s">
-        <v>417</v>
-      </c>
       <c r="E12" t="s">
         <v>150</v>
       </c>
@@ -7876,13 +8044,13 @@
         <v>150</v>
       </c>
       <c r="G12" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -7905,18 +8073,18 @@
         <v>150</v>
       </c>
       <c r="G13" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B14" t="s">
         <v>211</v>
@@ -7925,7 +8093,7 @@
         <v>387</v>
       </c>
       <c r="D14" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E14" t="s">
         <v>150</v>
@@ -7934,27 +8102,27 @@
         <v>150</v>
       </c>
       <c r="G14" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H14">
         <v>0</v>
       </c>
       <c r="I14" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
+        <v>419</v>
+      </c>
+      <c r="B15" t="s">
         <v>420</v>
       </c>
-      <c r="B15" t="s">
-        <v>421</v>
-      </c>
       <c r="C15" t="s">
         <v>387</v>
       </c>
       <c r="D15" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E15" t="s">
         <v>150</v>
@@ -7963,27 +8131,27 @@
         <v>150</v>
       </c>
       <c r="G15" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H15">
         <v>0</v>
       </c>
       <c r="I15" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
+        <v>421</v>
+      </c>
+      <c r="B16" t="s">
+        <v>517</v>
+      </c>
+      <c r="C16" t="s">
+        <v>516</v>
+      </c>
+      <c r="D16" t="s">
         <v>422</v>
-      </c>
-      <c r="B16" t="s">
-        <v>519</v>
-      </c>
-      <c r="C16" t="s">
-        <v>518</v>
-      </c>
-      <c r="D16" t="s">
-        <v>423</v>
       </c>
       <c r="E16" t="s">
         <v>150</v>
@@ -7998,21 +8166,21 @@
         <v>1</v>
       </c>
       <c r="I16" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B17" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="C17" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D17" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E17" t="s">
         <v>150</v>
@@ -8027,21 +8195,21 @@
         <v>1</v>
       </c>
       <c r="I17" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B18" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="C18" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D18" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E18" t="s">
         <v>150</v>
@@ -8056,21 +8224,21 @@
         <v>1</v>
       </c>
       <c r="I18" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B19" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="C19" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D19" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E19" t="s">
         <v>150</v>
@@ -8085,21 +8253,21 @@
         <v>1</v>
       </c>
       <c r="I19" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B20" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="C20" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D20" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E20" t="s">
         <v>150</v>
@@ -8114,21 +8282,21 @@
         <v>1</v>
       </c>
       <c r="I20" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B21" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C21" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D21" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E21" t="s">
         <v>150</v>
@@ -8143,21 +8311,21 @@
         <v>1</v>
       </c>
       <c r="I21" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B22" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="C22" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D22" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E22" t="s">
         <v>150</v>
@@ -8172,21 +8340,21 @@
         <v>1</v>
       </c>
       <c r="I22" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B23" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C23" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D23" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E23" t="s">
         <v>150</v>
@@ -8201,21 +8369,21 @@
         <v>1</v>
       </c>
       <c r="I23" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
+        <v>430</v>
+      </c>
+      <c r="B24" t="s">
         <v>431</v>
       </c>
-      <c r="B24" t="s">
-        <v>432</v>
-      </c>
       <c r="C24" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D24" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E24" t="s">
         <v>150</v>
@@ -8230,21 +8398,21 @@
         <v>1</v>
       </c>
       <c r="I24" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B25" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="C25" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D25" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E25" t="s">
         <v>150</v>
@@ -8259,21 +8427,21 @@
         <v>1</v>
       </c>
       <c r="I25" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B26" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C26" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D26" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E26" t="s">
         <v>150</v>
@@ -8288,21 +8456,21 @@
         <v>1</v>
       </c>
       <c r="I26" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B27" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C27" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D27" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E27" t="s">
         <v>150</v>
@@ -8317,21 +8485,21 @@
         <v>1</v>
       </c>
       <c r="I27" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B28" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C28" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D28" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E28" t="s">
         <v>150</v>
@@ -8346,21 +8514,21 @@
         <v>1</v>
       </c>
       <c r="I28" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B29" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C29" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D29" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E29" t="s">
         <v>150</v>
@@ -8375,21 +8543,21 @@
         <v>1</v>
       </c>
       <c r="I29" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B30" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C30" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D30" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E30" t="s">
         <v>150</v>
@@ -8404,21 +8572,21 @@
         <v>1</v>
       </c>
       <c r="I30" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B31" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C31" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D31" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E31" t="s">
         <v>150</v>
@@ -8433,21 +8601,21 @@
         <v>1</v>
       </c>
       <c r="I31" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B32" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="C32" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D32" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E32" t="s">
         <v>150</v>
@@ -8462,21 +8630,21 @@
         <v>1</v>
       </c>
       <c r="I32" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="33" spans="1:9">
       <c r="A33" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B33" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C33" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D33" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E33" t="s">
         <v>150</v>
@@ -8491,21 +8659,21 @@
         <v>1</v>
       </c>
       <c r="I33" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="34" spans="1:9">
       <c r="A34" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B34" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="C34" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D34" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E34" t="s">
         <v>150</v>
@@ -8520,21 +8688,21 @@
         <v>1</v>
       </c>
       <c r="I34" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="35" spans="1:9">
       <c r="A35" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B35" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C35" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D35" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E35" t="s">
         <v>150</v>
@@ -8549,21 +8717,21 @@
         <v>1</v>
       </c>
       <c r="I35" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B36" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C36" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D36" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E36" t="s">
         <v>150</v>
@@ -8578,21 +8746,21 @@
         <v>1</v>
       </c>
       <c r="I36" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="37" spans="1:9">
       <c r="A37" t="s">
+        <v>444</v>
+      </c>
+      <c r="B37" t="s">
         <v>445</v>
       </c>
-      <c r="B37" t="s">
-        <v>446</v>
-      </c>
       <c r="C37" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D37" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E37" t="s">
         <v>150</v>
@@ -8607,21 +8775,21 @@
         <v>1</v>
       </c>
       <c r="I37" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" t="s">
+        <v>446</v>
+      </c>
+      <c r="B38" t="s">
         <v>447</v>
       </c>
-      <c r="B38" t="s">
-        <v>448</v>
-      </c>
       <c r="C38" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D38" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E38" t="s">
         <v>150</v>
@@ -8636,21 +8804,21 @@
         <v>1</v>
       </c>
       <c r="I38" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="39" spans="1:9">
       <c r="A39" t="s">
+        <v>448</v>
+      </c>
+      <c r="B39" t="s">
         <v>449</v>
       </c>
-      <c r="B39" t="s">
-        <v>450</v>
-      </c>
       <c r="C39" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D39" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E39" t="s">
         <v>150</v>
@@ -8665,21 +8833,21 @@
         <v>1</v>
       </c>
       <c r="I39" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B40" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C40" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D40" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E40" t="s">
         <v>150</v>
@@ -8694,21 +8862,21 @@
         <v>1</v>
       </c>
       <c r="I40" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" t="s">
+        <v>451</v>
+      </c>
+      <c r="B41" t="s">
         <v>452</v>
       </c>
-      <c r="B41" t="s">
-        <v>453</v>
-      </c>
       <c r="C41" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D41" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E41" t="s">
         <v>150</v>
@@ -8723,21 +8891,21 @@
         <v>1</v>
       </c>
       <c r="I41" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" t="s">
+        <v>453</v>
+      </c>
+      <c r="B42" t="s">
         <v>454</v>
       </c>
-      <c r="B42" t="s">
-        <v>455</v>
-      </c>
       <c r="C42" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D42" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E42" t="s">
         <v>150</v>
@@ -8752,21 +8920,21 @@
         <v>1</v>
       </c>
       <c r="I42" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
+        <v>455</v>
+      </c>
+      <c r="B43" t="s">
         <v>456</v>
       </c>
-      <c r="B43" t="s">
-        <v>457</v>
-      </c>
       <c r="C43" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D43" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E43" t="s">
         <v>150</v>
@@ -8781,21 +8949,21 @@
         <v>1</v>
       </c>
       <c r="I43" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" t="s">
+        <v>457</v>
+      </c>
+      <c r="B44" t="s">
         <v>458</v>
       </c>
-      <c r="B44" t="s">
-        <v>459</v>
-      </c>
       <c r="C44" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D44" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E44" t="s">
         <v>150</v>
@@ -8810,21 +8978,21 @@
         <v>1</v>
       </c>
       <c r="I44" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" t="s">
+        <v>459</v>
+      </c>
+      <c r="B45" t="s">
         <v>460</v>
       </c>
-      <c r="B45" t="s">
-        <v>461</v>
-      </c>
       <c r="C45" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D45" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E45" t="s">
         <v>150</v>
@@ -8839,21 +9007,21 @@
         <v>1</v>
       </c>
       <c r="I45" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" t="s">
+        <v>461</v>
+      </c>
+      <c r="B46" t="s">
         <v>462</v>
       </c>
-      <c r="B46" t="s">
-        <v>463</v>
-      </c>
       <c r="C46" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D46" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E46" t="s">
         <v>150</v>
@@ -8868,21 +9036,21 @@
         <v>1</v>
       </c>
       <c r="I46" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" t="s">
+        <v>463</v>
+      </c>
+      <c r="B47" t="s">
         <v>464</v>
       </c>
-      <c r="B47" t="s">
-        <v>465</v>
-      </c>
       <c r="C47" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D47" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E47" t="s">
         <v>150</v>
@@ -8897,21 +9065,21 @@
         <v>1</v>
       </c>
       <c r="I47" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" t="s">
+        <v>465</v>
+      </c>
+      <c r="B48" t="s">
         <v>466</v>
       </c>
-      <c r="B48" t="s">
-        <v>467</v>
-      </c>
       <c r="C48" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D48" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E48" t="s">
         <v>150</v>
@@ -8926,21 +9094,21 @@
         <v>1</v>
       </c>
       <c r="I48" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" t="s">
+        <v>467</v>
+      </c>
+      <c r="B49" t="s">
         <v>468</v>
       </c>
-      <c r="B49" t="s">
-        <v>469</v>
-      </c>
       <c r="C49" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D49" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E49" t="s">
         <v>150</v>
@@ -8955,21 +9123,21 @@
         <v>1</v>
       </c>
       <c r="I49" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
+        <v>469</v>
+      </c>
+      <c r="B50" t="s">
         <v>470</v>
       </c>
-      <c r="B50" t="s">
-        <v>471</v>
-      </c>
       <c r="C50" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D50" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E50" t="s">
         <v>150</v>
@@ -8984,21 +9152,21 @@
         <v>1</v>
       </c>
       <c r="I50" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B51" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="C51" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D51" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E51" t="s">
         <v>150</v>
@@ -9013,21 +9181,21 @@
         <v>1</v>
       </c>
       <c r="I51" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="52" spans="1:9">
       <c r="A52" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B52" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C52" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D52" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E52" t="s">
         <v>150</v>
@@ -9042,21 +9210,21 @@
         <v>1</v>
       </c>
       <c r="I52" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="53" spans="1:9">
       <c r="A53" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B53" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="C53" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D53" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E53" t="s">
         <v>150</v>
@@ -9071,21 +9239,21 @@
         <v>1</v>
       </c>
       <c r="I53" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="54" spans="1:9">
       <c r="A54" t="s">
+        <v>474</v>
+      </c>
+      <c r="B54" t="s">
         <v>475</v>
       </c>
-      <c r="B54" t="s">
-        <v>476</v>
-      </c>
       <c r="C54" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D54" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E54" t="s">
         <v>150</v>
@@ -9100,21 +9268,21 @@
         <v>1</v>
       </c>
       <c r="I54" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="55" spans="1:9">
       <c r="A55" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B55" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C55" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D55" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E55" t="s">
         <v>150</v>
@@ -9129,21 +9297,21 @@
         <v>1</v>
       </c>
       <c r="I55" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="56" spans="1:9">
       <c r="A56" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B56" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="C56" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D56" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E56" t="s">
         <v>150</v>
@@ -9158,21 +9326,21 @@
         <v>1</v>
       </c>
       <c r="I56" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="57" spans="1:9">
       <c r="A57" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B57" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C57" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D57" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E57" t="s">
         <v>150</v>
@@ -9187,21 +9355,21 @@
         <v>0</v>
       </c>
       <c r="I57" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="58" spans="1:9">
       <c r="A58" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B58" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="C58" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D58" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E58" t="s">
         <v>150</v>
@@ -9216,21 +9384,21 @@
         <v>0</v>
       </c>
       <c r="I58" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="59" spans="1:9">
       <c r="A59" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B59" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="C59" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D59" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E59" t="s">
         <v>150</v>
@@ -9245,21 +9413,21 @@
         <v>0</v>
       </c>
       <c r="I59" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="60" spans="1:9">
       <c r="A60" t="s">
+        <v>481</v>
+      </c>
+      <c r="B60" t="s">
         <v>482</v>
       </c>
-      <c r="B60" t="s">
-        <v>483</v>
-      </c>
       <c r="C60" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D60" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E60" t="s">
         <v>150</v>
@@ -9274,21 +9442,21 @@
         <v>0</v>
       </c>
       <c r="I60" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="61" spans="1:9">
       <c r="A61" t="s">
+        <v>483</v>
+      </c>
+      <c r="B61" t="s">
         <v>484</v>
       </c>
-      <c r="B61" t="s">
-        <v>485</v>
-      </c>
       <c r="C61" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D61" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E61" t="s">
         <v>150</v>
@@ -9303,21 +9471,21 @@
         <v>0</v>
       </c>
       <c r="I61" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="62" spans="1:9">
       <c r="A62" t="s">
+        <v>485</v>
+      </c>
+      <c r="B62" t="s">
         <v>486</v>
       </c>
-      <c r="B62" t="s">
-        <v>487</v>
-      </c>
       <c r="C62" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D62" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E62" t="s">
         <v>150</v>
@@ -9332,21 +9500,21 @@
         <v>1</v>
       </c>
       <c r="I62" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="63" spans="1:9">
       <c r="A63" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B63" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="C63" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D63" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E63" t="s">
         <v>150</v>
@@ -9361,21 +9529,21 @@
         <v>1</v>
       </c>
       <c r="I63" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="64" spans="1:9">
       <c r="A64" t="s">
+        <v>488</v>
+      </c>
+      <c r="B64" t="s">
+        <v>510</v>
+      </c>
+      <c r="C64" t="s">
+        <v>515</v>
+      </c>
+      <c r="D64" t="s">
         <v>489</v>
-      </c>
-      <c r="B64" t="s">
-        <v>512</v>
-      </c>
-      <c r="C64" t="s">
-        <v>517</v>
-      </c>
-      <c r="D64" t="s">
-        <v>490</v>
       </c>
       <c r="E64" t="s">
         <v>150</v>
@@ -9390,21 +9558,21 @@
         <v>1</v>
       </c>
       <c r="I64" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="65" spans="1:9">
       <c r="A65" t="s">
+        <v>490</v>
+      </c>
+      <c r="B65" t="s">
+        <v>506</v>
+      </c>
+      <c r="C65" t="s">
+        <v>515</v>
+      </c>
+      <c r="D65" t="s">
         <v>491</v>
-      </c>
-      <c r="B65" t="s">
-        <v>508</v>
-      </c>
-      <c r="C65" t="s">
-        <v>517</v>
-      </c>
-      <c r="D65" t="s">
-        <v>492</v>
       </c>
       <c r="E65" t="s">
         <v>150</v>
@@ -9419,21 +9587,21 @@
         <v>1</v>
       </c>
       <c r="I65" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="66" spans="1:9">
       <c r="A66" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B66" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="C66" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D66" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="E66" t="s">
         <v>150</v>
@@ -9448,21 +9616,21 @@
         <v>1</v>
       </c>
       <c r="I66" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="67" spans="1:9">
       <c r="A67" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B67" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C67" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D67" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="E67" t="s">
         <v>150</v>
@@ -9477,21 +9645,21 @@
         <v>1</v>
       </c>
       <c r="I67" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="68" spans="1:9">
       <c r="A68" t="s">
+        <v>494</v>
+      </c>
+      <c r="B68" t="s">
         <v>495</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
+        <v>515</v>
+      </c>
+      <c r="D68" t="s">
         <v>496</v>
-      </c>
-      <c r="C68" t="s">
-        <v>517</v>
-      </c>
-      <c r="D68" t="s">
-        <v>497</v>
       </c>
       <c r="E68" t="s">
         <v>150</v>
@@ -9506,21 +9674,21 @@
         <v>0</v>
       </c>
       <c r="I68" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="69" spans="1:9">
       <c r="A69" t="s">
+        <v>497</v>
+      </c>
+      <c r="B69" t="s">
         <v>498</v>
       </c>
-      <c r="B69" t="s">
-        <v>499</v>
-      </c>
       <c r="C69" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D69" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E69" t="s">
         <v>150</v>
@@ -9535,21 +9703,21 @@
         <v>0</v>
       </c>
       <c r="I69" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="70" spans="1:9">
       <c r="A70" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B70" t="s">
+        <v>513</v>
+      </c>
+      <c r="C70" t="s">
         <v>515</v>
       </c>
-      <c r="C70" t="s">
-        <v>517</v>
-      </c>
       <c r="D70" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E70" t="s">
         <v>150</v>
@@ -9564,21 +9732,21 @@
         <v>0</v>
       </c>
       <c r="I70" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="71" spans="1:9">
       <c r="A71" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B71" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="C71" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D71" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E71" t="s">
         <v>150</v>
@@ -9593,21 +9761,21 @@
         <v>0</v>
       </c>
       <c r="I71" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="72" spans="1:9">
       <c r="A72" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B72" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C72" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D72" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E72" t="s">
         <v>150</v>
@@ -9622,21 +9790,21 @@
         <v>0</v>
       </c>
       <c r="I72" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="73" spans="1:9">
       <c r="A73" t="s">
+        <v>502</v>
+      </c>
+      <c r="B73" t="s">
+        <v>543</v>
+      </c>
+      <c r="C73" t="s">
+        <v>515</v>
+      </c>
+      <c r="D73" t="s">
         <v>503</v>
-      </c>
-      <c r="B73" t="s">
-        <v>545</v>
-      </c>
-      <c r="C73" t="s">
-        <v>517</v>
-      </c>
-      <c r="D73" t="s">
-        <v>505</v>
       </c>
       <c r="E73" t="s">
         <v>150</v>
@@ -9651,21 +9819,21 @@
         <v>1</v>
       </c>
       <c r="I73" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="74" spans="1:9">
       <c r="A74" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="B74" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="C74" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D74" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="E74" t="s">
         <v>150</v>
@@ -9680,21 +9848,21 @@
         <v>1</v>
       </c>
       <c r="I74" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="75" spans="1:9">
       <c r="A75" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B75" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="C75" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D75" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="E75" t="s">
         <v>150</v>
@@ -9709,7 +9877,7 @@
         <v>1</v>
       </c>
       <c r="I75" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
   </sheetData>
@@ -9719,162 +9887,183 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41309215-EB4C-48B3-A3D7-89B6FA6A2DA4}">
-  <dimension ref="A1:I68"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1936B2BD-9EC2-4ACF-BEDD-4E61EE334CEE}">
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="112.5703125" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col min="2" max="2" width="81.42578125" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="21.85546875" customWidth="1"/>
     <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" customWidth="1"/>
     <col min="8" max="8" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>544</v>
+      </c>
+      <c r="B2" t="s">
+        <v>545</v>
+      </c>
+      <c r="C2" t="s">
+        <v>387</v>
+      </c>
+      <c r="D2" t="s">
+        <v>400</v>
+      </c>
+      <c r="E2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G2" t="s">
+        <v>387</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>401</v>
+      </c>
+      <c r="B3" t="s">
         <v>402</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C3" t="s">
+        <v>387</v>
+      </c>
+      <c r="D3" t="s">
+        <v>400</v>
+      </c>
+      <c r="E3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G3" t="s">
+        <v>387</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>547</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="C4" t="s">
+        <v>387</v>
+      </c>
+      <c r="D4" t="s">
+        <v>558</v>
+      </c>
+      <c r="E4" t="s">
+        <v>150</v>
+      </c>
+      <c r="F4" t="s">
+        <v>150</v>
+      </c>
+      <c r="G4" t="s">
+        <v>387</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>557</v>
+      </c>
+      <c r="B5" t="s">
+        <v>564</v>
+      </c>
+      <c r="C5" t="s">
+        <v>387</v>
+      </c>
+      <c r="D5" t="s">
+        <v>558</v>
+      </c>
+      <c r="E5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F5" t="s">
+        <v>150</v>
+      </c>
+      <c r="G5" t="s">
+        <v>387</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
         <v>403</v>
       </c>
-      <c r="D1" t="s">
-        <v>401</v>
-      </c>
-      <c r="E1" t="s">
-        <v>150</v>
-      </c>
-      <c r="F1" t="s">
-        <v>150</v>
-      </c>
-      <c r="G1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H1">
-        <v>0</v>
-      </c>
-      <c r="I1" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
+      <c r="B6" t="s">
         <v>404</v>
       </c>
-      <c r="B2" t="s">
-        <v>405</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C6" t="s">
+        <v>387</v>
+      </c>
+      <c r="D6" t="s">
         <v>192</v>
       </c>
-      <c r="E2" t="s">
-        <v>150</v>
-      </c>
-      <c r="F2" t="s">
-        <v>150</v>
-      </c>
-      <c r="G2" t="s">
-        <v>197</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>406</v>
-      </c>
-      <c r="B3" t="s">
-        <v>407</v>
-      </c>
-      <c r="D3" t="s">
-        <v>408</v>
-      </c>
-      <c r="E3" t="s">
-        <v>150</v>
-      </c>
-      <c r="F3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G3" t="s">
-        <v>197</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>409</v>
-      </c>
-      <c r="B4" t="s">
-        <v>410</v>
-      </c>
-      <c r="D4" t="s">
-        <v>408</v>
-      </c>
-      <c r="E4" t="s">
-        <v>150</v>
-      </c>
-      <c r="F4" t="s">
-        <v>150</v>
-      </c>
-      <c r="G4" t="s">
-        <v>197</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>411</v>
-      </c>
-      <c r="B5" t="s">
-        <v>412</v>
-      </c>
-      <c r="D5" t="s">
-        <v>192</v>
-      </c>
-      <c r="E5" t="s">
-        <v>150</v>
-      </c>
-      <c r="F5" t="s">
-        <v>150</v>
-      </c>
-      <c r="G5" t="s">
-        <v>197</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>413</v>
-      </c>
-      <c r="B6" t="s">
-        <v>414</v>
-      </c>
-      <c r="D6" t="s">
-        <v>408</v>
-      </c>
       <c r="E6" t="s">
         <v>150</v>
       </c>
@@ -9882,24 +10071,27 @@
         <v>150</v>
       </c>
       <c r="G6" t="s">
-        <v>197</v>
+        <v>387</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.75">
       <c r="A7" t="s">
-        <v>415</v>
-      </c>
-      <c r="B7" t="s">
-        <v>416</v>
+        <v>59</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="C7" t="s">
+        <v>392</v>
       </c>
       <c r="D7" t="s">
-        <v>417</v>
+        <v>585</v>
       </c>
       <c r="E7" t="s">
         <v>150</v>
@@ -9907,25 +10099,28 @@
       <c r="F7" t="s">
         <v>150</v>
       </c>
-      <c r="G7" t="s">
-        <v>197</v>
+      <c r="G7" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75">
       <c r="A8" t="s">
-        <v>397</v>
-      </c>
-      <c r="B8" t="s">
-        <v>398</v>
+        <v>60</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="C8" t="s">
+        <v>392</v>
       </c>
       <c r="D8" t="s">
-        <v>399</v>
+        <v>585</v>
       </c>
       <c r="E8" t="s">
         <v>150</v>
@@ -9933,25 +10128,28 @@
       <c r="F8" t="s">
         <v>150</v>
       </c>
-      <c r="G8" t="s">
-        <v>197</v>
+      <c r="G8" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.75">
       <c r="A9" t="s">
-        <v>418</v>
-      </c>
-      <c r="B9" t="s">
-        <v>211</v>
+        <v>61</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="C9" t="s">
+        <v>392</v>
       </c>
       <c r="D9" t="s">
-        <v>419</v>
+        <v>585</v>
       </c>
       <c r="E9" t="s">
         <v>150</v>
@@ -9959,25 +10157,28 @@
       <c r="F9" t="s">
         <v>150</v>
       </c>
-      <c r="G9" t="s">
-        <v>197</v>
+      <c r="G9" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.75">
       <c r="A10" t="s">
-        <v>420</v>
-      </c>
-      <c r="B10" t="s">
-        <v>421</v>
+        <v>62</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C10" t="s">
+        <v>392</v>
       </c>
       <c r="D10" t="s">
-        <v>408</v>
+        <v>585</v>
       </c>
       <c r="E10" t="s">
         <v>150</v>
@@ -9985,28 +10186,28 @@
       <c r="F10" t="s">
         <v>150</v>
       </c>
-      <c r="G10" t="s">
-        <v>197</v>
+      <c r="G10" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.75">
       <c r="A11" t="s">
-        <v>422</v>
-      </c>
-      <c r="B11" t="s">
-        <v>519</v>
+        <v>64</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>587</v>
       </c>
       <c r="C11" t="s">
-        <v>518</v>
+        <v>392</v>
       </c>
       <c r="D11" t="s">
-        <v>423</v>
+        <v>136</v>
       </c>
       <c r="E11" t="s">
         <v>150</v>
@@ -10014,28 +10215,28 @@
       <c r="F11" t="s">
         <v>150</v>
       </c>
-      <c r="G11" t="s">
-        <v>197</v>
+      <c r="G11" s="2" t="s">
+        <v>393</v>
       </c>
       <c r="H11">
         <v>1</v>
       </c>
       <c r="I11" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75">
       <c r="A12" t="s">
-        <v>424</v>
-      </c>
-      <c r="B12" t="s">
-        <v>520</v>
+        <v>57</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>593</v>
       </c>
       <c r="C12" t="s">
-        <v>518</v>
+        <v>392</v>
       </c>
       <c r="D12" t="s">
-        <v>423</v>
+        <v>559</v>
       </c>
       <c r="E12" t="s">
         <v>150</v>
@@ -10043,28 +10244,28 @@
       <c r="F12" t="s">
         <v>150</v>
       </c>
-      <c r="G12" t="s">
-        <v>197</v>
+      <c r="G12" s="2" t="s">
+        <v>393</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
       <c r="I12" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.75">
       <c r="A13" t="s">
-        <v>425</v>
-      </c>
-      <c r="B13" t="s">
-        <v>521</v>
+        <v>58</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>594</v>
       </c>
       <c r="C13" t="s">
-        <v>518</v>
+        <v>392</v>
       </c>
       <c r="D13" t="s">
-        <v>423</v>
+        <v>559</v>
       </c>
       <c r="E13" t="s">
         <v>150</v>
@@ -10072,28 +10273,28 @@
       <c r="F13" t="s">
         <v>150</v>
       </c>
-      <c r="G13" t="s">
-        <v>197</v>
+      <c r="G13" s="2" t="s">
+        <v>393</v>
       </c>
       <c r="H13">
         <v>1</v>
       </c>
       <c r="I13" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.75">
       <c r="A14" t="s">
-        <v>426</v>
-      </c>
-      <c r="B14" t="s">
-        <v>522</v>
+        <v>565</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>588</v>
       </c>
       <c r="C14" t="s">
-        <v>518</v>
-      </c>
-      <c r="D14" t="s">
-        <v>423</v>
+        <v>383</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>589</v>
       </c>
       <c r="E14" t="s">
         <v>150</v>
@@ -10101,28 +10302,28 @@
       <c r="F14" t="s">
         <v>150</v>
       </c>
-      <c r="G14" t="s">
-        <v>197</v>
+      <c r="G14" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H14">
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.75">
       <c r="A15" t="s">
-        <v>427</v>
-      </c>
-      <c r="B15" t="s">
-        <v>523</v>
+        <v>566</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>590</v>
       </c>
       <c r="C15" t="s">
-        <v>518</v>
+        <v>392</v>
       </c>
       <c r="D15" t="s">
-        <v>423</v>
+        <v>585</v>
       </c>
       <c r="E15" t="s">
         <v>150</v>
@@ -10130,28 +10331,28 @@
       <c r="F15" t="s">
         <v>150</v>
       </c>
-      <c r="G15" t="s">
-        <v>197</v>
+      <c r="G15" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H15">
         <v>1</v>
       </c>
       <c r="I15" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.75">
       <c r="A16" t="s">
-        <v>428</v>
-      </c>
-      <c r="B16" t="s">
-        <v>524</v>
+        <v>567</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>591</v>
       </c>
       <c r="C16" t="s">
-        <v>518</v>
+        <v>392</v>
       </c>
       <c r="D16" t="s">
-        <v>423</v>
+        <v>585</v>
       </c>
       <c r="E16" t="s">
         <v>150</v>
@@ -10159,28 +10360,28 @@
       <c r="F16" t="s">
         <v>150</v>
       </c>
-      <c r="G16" t="s">
-        <v>197</v>
+      <c r="G16" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H16">
         <v>1</v>
       </c>
       <c r="I16" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="15.75">
       <c r="A17" t="s">
-        <v>429</v>
-      </c>
-      <c r="B17" t="s">
-        <v>525</v>
+        <v>568</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>592</v>
       </c>
       <c r="C17" t="s">
-        <v>518</v>
+        <v>392</v>
       </c>
       <c r="D17" t="s">
-        <v>423</v>
+        <v>585</v>
       </c>
       <c r="E17" t="s">
         <v>150</v>
@@ -10188,28 +10389,28 @@
       <c r="F17" t="s">
         <v>150</v>
       </c>
-      <c r="G17" t="s">
-        <v>197</v>
+      <c r="G17" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H17">
         <v>1</v>
       </c>
       <c r="I17" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.75">
       <c r="A18" t="s">
-        <v>430</v>
+        <v>569</v>
       </c>
       <c r="B18" t="s">
-        <v>526</v>
+        <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D18" t="s">
-        <v>423</v>
+        <v>560</v>
       </c>
       <c r="E18" t="s">
         <v>150</v>
@@ -10217,25 +10418,28 @@
       <c r="F18" t="s">
         <v>150</v>
       </c>
-      <c r="G18" t="s">
-        <v>197</v>
+      <c r="G18" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H18">
         <v>1</v>
       </c>
       <c r="I18" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15.75">
       <c r="A19" t="s">
-        <v>431</v>
+        <v>570</v>
       </c>
       <c r="B19" t="s">
-        <v>432</v>
+        <v>607</v>
+      </c>
+      <c r="C19" t="s">
+        <v>383</v>
       </c>
       <c r="D19" t="s">
-        <v>423</v>
+        <v>139</v>
       </c>
       <c r="E19" t="s">
         <v>150</v>
@@ -10243,28 +10447,28 @@
       <c r="F19" t="s">
         <v>150</v>
       </c>
-      <c r="G19" t="s">
-        <v>197</v>
+      <c r="G19" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H19">
         <v>1</v>
       </c>
       <c r="I19" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="15.75">
       <c r="A20" t="s">
-        <v>433</v>
+        <v>571</v>
       </c>
       <c r="B20" t="s">
-        <v>527</v>
+        <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D20" t="s">
-        <v>423</v>
+        <v>608</v>
       </c>
       <c r="E20" t="s">
         <v>150</v>
@@ -10272,28 +10476,28 @@
       <c r="F20" t="s">
         <v>150</v>
       </c>
-      <c r="G20" t="s">
-        <v>197</v>
+      <c r="G20" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H20">
         <v>1</v>
       </c>
       <c r="I20" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="15.75">
       <c r="A21" t="s">
-        <v>434</v>
+        <v>572</v>
       </c>
       <c r="B21" t="s">
-        <v>528</v>
+        <v>606</v>
       </c>
       <c r="C21" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D21" t="s">
-        <v>423</v>
+        <v>605</v>
       </c>
       <c r="E21" t="s">
         <v>150</v>
@@ -10301,28 +10505,28 @@
       <c r="F21" t="s">
         <v>150</v>
       </c>
-      <c r="G21" t="s">
-        <v>197</v>
+      <c r="G21" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H21">
         <v>1</v>
       </c>
       <c r="I21" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="15.75">
       <c r="A22" t="s">
-        <v>435</v>
+        <v>573</v>
       </c>
       <c r="B22" t="s">
-        <v>529</v>
+        <v>604</v>
       </c>
       <c r="C22" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D22" t="s">
-        <v>423</v>
+        <v>144</v>
       </c>
       <c r="E22" t="s">
         <v>150</v>
@@ -10330,28 +10534,28 @@
       <c r="F22" t="s">
         <v>150</v>
       </c>
-      <c r="G22" t="s">
-        <v>197</v>
+      <c r="G22" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H22">
         <v>1</v>
       </c>
       <c r="I22" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="15.75">
       <c r="A23" t="s">
-        <v>436</v>
+        <v>574</v>
       </c>
       <c r="B23" t="s">
-        <v>530</v>
+        <v>603</v>
       </c>
       <c r="C23" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D23" t="s">
-        <v>423</v>
+        <v>609</v>
       </c>
       <c r="E23" t="s">
         <v>150</v>
@@ -10359,28 +10563,28 @@
       <c r="F23" t="s">
         <v>150</v>
       </c>
-      <c r="G23" t="s">
-        <v>197</v>
+      <c r="G23" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H23">
         <v>1</v>
       </c>
       <c r="I23" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="15.75">
       <c r="A24" t="s">
-        <v>437</v>
+        <v>561</v>
       </c>
       <c r="B24" t="s">
-        <v>531</v>
+        <v>602</v>
       </c>
       <c r="C24" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D24" t="s">
-        <v>423</v>
+        <v>610</v>
       </c>
       <c r="E24" t="s">
         <v>150</v>
@@ -10388,28 +10592,28 @@
       <c r="F24" t="s">
         <v>150</v>
       </c>
-      <c r="G24" t="s">
-        <v>197</v>
+      <c r="G24" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H24">
         <v>1</v>
       </c>
       <c r="I24" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15.75">
       <c r="A25" t="s">
-        <v>438</v>
+        <v>575</v>
       </c>
       <c r="B25" t="s">
-        <v>532</v>
+        <v>601</v>
       </c>
       <c r="C25" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D25" t="s">
-        <v>423</v>
+        <v>610</v>
       </c>
       <c r="E25" t="s">
         <v>150</v>
@@ -10417,28 +10621,28 @@
       <c r="F25" t="s">
         <v>150</v>
       </c>
-      <c r="G25" t="s">
-        <v>197</v>
+      <c r="G25" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H25">
         <v>1</v>
       </c>
       <c r="I25" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="15.75">
       <c r="A26" t="s">
-        <v>439</v>
+        <v>562</v>
       </c>
       <c r="B26" t="s">
-        <v>533</v>
+        <v>600</v>
       </c>
       <c r="C26" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D26" t="s">
-        <v>423</v>
+        <v>589</v>
       </c>
       <c r="E26" t="s">
         <v>150</v>
@@ -10446,28 +10650,28 @@
       <c r="F26" t="s">
         <v>150</v>
       </c>
-      <c r="G26" t="s">
-        <v>197</v>
+      <c r="G26" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H26">
         <v>1</v>
       </c>
       <c r="I26" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="15.75">
       <c r="A27" t="s">
-        <v>440</v>
+        <v>576</v>
       </c>
       <c r="B27" t="s">
-        <v>534</v>
+        <v>599</v>
       </c>
       <c r="C27" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D27" t="s">
-        <v>423</v>
+        <v>589</v>
       </c>
       <c r="E27" t="s">
         <v>150</v>
@@ -10475,28 +10679,28 @@
       <c r="F27" t="s">
         <v>150</v>
       </c>
-      <c r="G27" t="s">
-        <v>197</v>
+      <c r="G27" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H27">
         <v>1</v>
       </c>
       <c r="I27" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15.75">
       <c r="A28" t="s">
-        <v>441</v>
+        <v>577</v>
       </c>
       <c r="B28" t="s">
-        <v>535</v>
+        <v>598</v>
       </c>
       <c r="C28" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D28" t="s">
-        <v>423</v>
+        <v>611</v>
       </c>
       <c r="E28" t="s">
         <v>150</v>
@@ -10504,28 +10708,28 @@
       <c r="F28" t="s">
         <v>150</v>
       </c>
-      <c r="G28" t="s">
-        <v>197</v>
+      <c r="G28" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H28">
         <v>1</v>
       </c>
       <c r="I28" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15.75">
       <c r="A29" t="s">
-        <v>442</v>
+        <v>578</v>
       </c>
       <c r="B29" t="s">
-        <v>536</v>
+        <v>612</v>
       </c>
       <c r="C29" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D29" t="s">
-        <v>423</v>
+        <v>613</v>
       </c>
       <c r="E29" t="s">
         <v>150</v>
@@ -10533,28 +10737,28 @@
       <c r="F29" t="s">
         <v>150</v>
       </c>
-      <c r="G29" t="s">
-        <v>197</v>
+      <c r="G29" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H29">
         <v>1</v>
       </c>
       <c r="I29" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.75">
       <c r="A30" t="s">
-        <v>443</v>
+        <v>579</v>
       </c>
       <c r="B30" t="s">
-        <v>537</v>
+        <v>597</v>
       </c>
       <c r="C30" t="s">
-        <v>518</v>
+        <v>383</v>
       </c>
       <c r="D30" t="s">
-        <v>423</v>
+        <v>613</v>
       </c>
       <c r="E30" t="s">
         <v>150</v>
@@ -10562,28 +10766,28 @@
       <c r="F30" t="s">
         <v>150</v>
       </c>
-      <c r="G30" t="s">
-        <v>197</v>
+      <c r="G30" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H30">
         <v>1</v>
       </c>
       <c r="I30" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="15.75">
       <c r="A31" t="s">
-        <v>444</v>
+        <v>580</v>
       </c>
       <c r="B31" t="s">
-        <v>538</v>
+        <v>596</v>
       </c>
       <c r="C31" t="s">
-        <v>518</v>
+        <v>392</v>
       </c>
       <c r="D31" t="s">
-        <v>423</v>
+        <v>614</v>
       </c>
       <c r="E31" t="s">
         <v>150</v>
@@ -10591,25 +10795,28 @@
       <c r="F31" t="s">
         <v>150</v>
       </c>
-      <c r="G31" t="s">
-        <v>197</v>
+      <c r="G31" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="15.75">
       <c r="A32" t="s">
-        <v>445</v>
+        <v>581</v>
       </c>
       <c r="B32" t="s">
-        <v>446</v>
+        <v>595</v>
+      </c>
+      <c r="C32" t="s">
+        <v>392</v>
       </c>
       <c r="D32" t="s">
-        <v>423</v>
+        <v>136</v>
       </c>
       <c r="E32" t="s">
         <v>150</v>
@@ -10617,998 +10824,14 @@
       <c r="F32" t="s">
         <v>150</v>
       </c>
-      <c r="G32" t="s">
-        <v>197</v>
+      <c r="G32" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="H32">
         <v>1</v>
       </c>
       <c r="I32" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9">
-      <c r="A33" t="s">
-        <v>447</v>
-      </c>
-      <c r="B33" t="s">
-        <v>448</v>
-      </c>
-      <c r="D33" t="s">
-        <v>408</v>
-      </c>
-      <c r="E33" t="s">
-        <v>150</v>
-      </c>
-      <c r="F33" t="s">
-        <v>150</v>
-      </c>
-      <c r="G33" t="s">
-        <v>197</v>
-      </c>
-      <c r="H33">
-        <v>1</v>
-      </c>
-      <c r="I33" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9">
-      <c r="A34" t="s">
-        <v>449</v>
-      </c>
-      <c r="B34" t="s">
-        <v>450</v>
-      </c>
-      <c r="D34" t="s">
-        <v>408</v>
-      </c>
-      <c r="E34" t="s">
-        <v>150</v>
-      </c>
-      <c r="F34" t="s">
-        <v>150</v>
-      </c>
-      <c r="G34" t="s">
-        <v>197</v>
-      </c>
-      <c r="H34">
-        <v>1</v>
-      </c>
-      <c r="I34" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9">
-      <c r="A35" t="s">
-        <v>451</v>
-      </c>
-      <c r="B35" t="s">
-        <v>539</v>
-      </c>
-      <c r="C35" t="s">
-        <v>518</v>
-      </c>
-      <c r="D35" t="s">
-        <v>423</v>
-      </c>
-      <c r="E35" t="s">
-        <v>150</v>
-      </c>
-      <c r="F35" t="s">
-        <v>150</v>
-      </c>
-      <c r="G35" t="s">
-        <v>197</v>
-      </c>
-      <c r="H35">
-        <v>1</v>
-      </c>
-      <c r="I35" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9">
-      <c r="A36" t="s">
-        <v>452</v>
-      </c>
-      <c r="B36" t="s">
-        <v>453</v>
-      </c>
-      <c r="D36" t="s">
-        <v>423</v>
-      </c>
-      <c r="E36" t="s">
-        <v>150</v>
-      </c>
-      <c r="F36" t="s">
-        <v>150</v>
-      </c>
-      <c r="G36" t="s">
-        <v>197</v>
-      </c>
-      <c r="H36">
-        <v>1</v>
-      </c>
-      <c r="I36" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9">
-      <c r="A37" t="s">
-        <v>454</v>
-      </c>
-      <c r="B37" t="s">
-        <v>455</v>
-      </c>
-      <c r="D37" t="s">
-        <v>408</v>
-      </c>
-      <c r="E37" t="s">
-        <v>150</v>
-      </c>
-      <c r="F37" t="s">
-        <v>150</v>
-      </c>
-      <c r="G37" t="s">
-        <v>197</v>
-      </c>
-      <c r="H37">
-        <v>1</v>
-      </c>
-      <c r="I37" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9">
-      <c r="A38" t="s">
-        <v>456</v>
-      </c>
-      <c r="B38" t="s">
-        <v>457</v>
-      </c>
-      <c r="D38" t="s">
-        <v>423</v>
-      </c>
-      <c r="E38" t="s">
-        <v>150</v>
-      </c>
-      <c r="F38" t="s">
-        <v>150</v>
-      </c>
-      <c r="G38" t="s">
-        <v>197</v>
-      </c>
-      <c r="H38">
-        <v>1</v>
-      </c>
-      <c r="I38" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9">
-      <c r="A39" t="s">
-        <v>458</v>
-      </c>
-      <c r="B39" t="s">
-        <v>459</v>
-      </c>
-      <c r="D39" t="s">
-        <v>408</v>
-      </c>
-      <c r="E39" t="s">
-        <v>150</v>
-      </c>
-      <c r="F39" t="s">
-        <v>150</v>
-      </c>
-      <c r="G39" t="s">
-        <v>197</v>
-      </c>
-      <c r="H39">
-        <v>1</v>
-      </c>
-      <c r="I39" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9">
-      <c r="A40" t="s">
-        <v>460</v>
-      </c>
-      <c r="B40" t="s">
-        <v>461</v>
-      </c>
-      <c r="D40" t="s">
-        <v>423</v>
-      </c>
-      <c r="E40" t="s">
-        <v>150</v>
-      </c>
-      <c r="F40" t="s">
-        <v>150</v>
-      </c>
-      <c r="G40" t="s">
-        <v>197</v>
-      </c>
-      <c r="H40">
-        <v>1</v>
-      </c>
-      <c r="I40" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9">
-      <c r="A41" t="s">
-        <v>462</v>
-      </c>
-      <c r="B41" t="s">
-        <v>463</v>
-      </c>
-      <c r="D41" t="s">
-        <v>408</v>
-      </c>
-      <c r="E41" t="s">
-        <v>150</v>
-      </c>
-      <c r="F41" t="s">
-        <v>150</v>
-      </c>
-      <c r="G41" t="s">
-        <v>197</v>
-      </c>
-      <c r="H41">
-        <v>1</v>
-      </c>
-      <c r="I41" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9">
-      <c r="A42" t="s">
-        <v>464</v>
-      </c>
-      <c r="B42" t="s">
-        <v>465</v>
-      </c>
-      <c r="D42" t="s">
-        <v>423</v>
-      </c>
-      <c r="E42" t="s">
-        <v>150</v>
-      </c>
-      <c r="F42" t="s">
-        <v>150</v>
-      </c>
-      <c r="G42" t="s">
-        <v>197</v>
-      </c>
-      <c r="H42">
-        <v>1</v>
-      </c>
-      <c r="I42" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9">
-      <c r="A43" t="s">
-        <v>466</v>
-      </c>
-      <c r="B43" t="s">
-        <v>467</v>
-      </c>
-      <c r="D43" t="s">
-        <v>423</v>
-      </c>
-      <c r="E43" t="s">
-        <v>150</v>
-      </c>
-      <c r="F43" t="s">
-        <v>150</v>
-      </c>
-      <c r="G43" t="s">
-        <v>197</v>
-      </c>
-      <c r="H43">
-        <v>1</v>
-      </c>
-      <c r="I43" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9">
-      <c r="A44" t="s">
-        <v>468</v>
-      </c>
-      <c r="B44" t="s">
-        <v>469</v>
-      </c>
-      <c r="D44" t="s">
-        <v>408</v>
-      </c>
-      <c r="E44" t="s">
-        <v>150</v>
-      </c>
-      <c r="F44" t="s">
-        <v>150</v>
-      </c>
-      <c r="G44" t="s">
-        <v>197</v>
-      </c>
-      <c r="H44">
-        <v>1</v>
-      </c>
-      <c r="I44" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9">
-      <c r="A45" t="s">
-        <v>470</v>
-      </c>
-      <c r="B45" t="s">
-        <v>471</v>
-      </c>
-      <c r="D45" t="s">
-        <v>408</v>
-      </c>
-      <c r="E45" t="s">
-        <v>150</v>
-      </c>
-      <c r="F45" t="s">
-        <v>150</v>
-      </c>
-      <c r="G45" t="s">
-        <v>197</v>
-      </c>
-      <c r="H45">
-        <v>1</v>
-      </c>
-      <c r="I45" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9">
-      <c r="A46" t="s">
-        <v>472</v>
-      </c>
-      <c r="B46" t="s">
-        <v>540</v>
-      </c>
-      <c r="C46" t="s">
-        <v>518</v>
-      </c>
-      <c r="D46" t="s">
-        <v>423</v>
-      </c>
-      <c r="E46" t="s">
-        <v>150</v>
-      </c>
-      <c r="F46" t="s">
-        <v>150</v>
-      </c>
-      <c r="G46" t="s">
-        <v>197</v>
-      </c>
-      <c r="H46">
-        <v>1</v>
-      </c>
-      <c r="I46" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9">
-      <c r="A47" t="s">
-        <v>473</v>
-      </c>
-      <c r="B47" t="s">
-        <v>541</v>
-      </c>
-      <c r="C47" t="s">
-        <v>518</v>
-      </c>
-      <c r="D47" t="s">
-        <v>423</v>
-      </c>
-      <c r="E47" t="s">
-        <v>150</v>
-      </c>
-      <c r="F47" t="s">
-        <v>150</v>
-      </c>
-      <c r="G47" t="s">
-        <v>197</v>
-      </c>
-      <c r="H47">
-        <v>1</v>
-      </c>
-      <c r="I47" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9">
-      <c r="A48" t="s">
-        <v>474</v>
-      </c>
-      <c r="B48" t="s">
-        <v>542</v>
-      </c>
-      <c r="C48" t="s">
-        <v>518</v>
-      </c>
-      <c r="D48" t="s">
-        <v>423</v>
-      </c>
-      <c r="E48" t="s">
-        <v>150</v>
-      </c>
-      <c r="F48" t="s">
-        <v>150</v>
-      </c>
-      <c r="G48" t="s">
-        <v>197</v>
-      </c>
-      <c r="H48">
-        <v>1</v>
-      </c>
-      <c r="I48" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9">
-      <c r="A49" t="s">
-        <v>475</v>
-      </c>
-      <c r="B49" t="s">
-        <v>476</v>
-      </c>
-      <c r="D49" t="s">
-        <v>423</v>
-      </c>
-      <c r="E49" t="s">
-        <v>150</v>
-      </c>
-      <c r="F49" t="s">
-        <v>150</v>
-      </c>
-      <c r="G49" t="s">
-        <v>197</v>
-      </c>
-      <c r="H49">
-        <v>1</v>
-      </c>
-      <c r="I49" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9">
-      <c r="A50" t="s">
-        <v>477</v>
-      </c>
-      <c r="B50" t="s">
-        <v>543</v>
-      </c>
-      <c r="C50" t="s">
-        <v>518</v>
-      </c>
-      <c r="D50" t="s">
-        <v>423</v>
-      </c>
-      <c r="E50" t="s">
-        <v>150</v>
-      </c>
-      <c r="F50" t="s">
-        <v>150</v>
-      </c>
-      <c r="G50" t="s">
-        <v>197</v>
-      </c>
-      <c r="H50">
-        <v>1</v>
-      </c>
-      <c r="I50" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9">
-      <c r="A51" t="s">
-        <v>478</v>
-      </c>
-      <c r="B51" t="s">
-        <v>544</v>
-      </c>
-      <c r="C51" t="s">
-        <v>518</v>
-      </c>
-      <c r="D51" t="s">
-        <v>423</v>
-      </c>
-      <c r="E51" t="s">
-        <v>150</v>
-      </c>
-      <c r="F51" t="s">
-        <v>150</v>
-      </c>
-      <c r="G51" t="s">
-        <v>197</v>
-      </c>
-      <c r="H51">
-        <v>1</v>
-      </c>
-      <c r="I51" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9">
-      <c r="A52" t="s">
-        <v>479</v>
-      </c>
-      <c r="B52" t="s">
-        <v>507</v>
-      </c>
-      <c r="C52" t="s">
-        <v>517</v>
-      </c>
-      <c r="E52" t="s">
-        <v>150</v>
-      </c>
-      <c r="F52" t="s">
-        <v>150</v>
-      </c>
-      <c r="G52" t="s">
-        <v>197</v>
-      </c>
-      <c r="H52">
-        <v>0</v>
-      </c>
-      <c r="I52" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9">
-      <c r="A53" t="s">
-        <v>480</v>
-      </c>
-      <c r="B53" t="s">
-        <v>511</v>
-      </c>
-      <c r="C53" t="s">
-        <v>517</v>
-      </c>
-      <c r="D53" t="s">
-        <v>408</v>
-      </c>
-      <c r="E53" t="s">
-        <v>150</v>
-      </c>
-      <c r="F53" t="s">
-        <v>150</v>
-      </c>
-      <c r="G53" t="s">
-        <v>197</v>
-      </c>
-      <c r="H53">
-        <v>0</v>
-      </c>
-      <c r="I53" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9">
-      <c r="A54" t="s">
-        <v>481</v>
-      </c>
-      <c r="B54" t="s">
-        <v>506</v>
-      </c>
-      <c r="C54" t="s">
-        <v>517</v>
-      </c>
-      <c r="D54" t="s">
-        <v>408</v>
-      </c>
-      <c r="E54" t="s">
-        <v>150</v>
-      </c>
-      <c r="F54" t="s">
-        <v>150</v>
-      </c>
-      <c r="G54" t="s">
-        <v>197</v>
-      </c>
-      <c r="H54">
-        <v>0</v>
-      </c>
-      <c r="I54" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9">
-      <c r="A55" t="s">
-        <v>482</v>
-      </c>
-      <c r="B55" t="s">
-        <v>483</v>
-      </c>
-      <c r="C55" t="s">
-        <v>517</v>
-      </c>
-      <c r="D55" t="s">
-        <v>419</v>
-      </c>
-      <c r="E55" t="s">
-        <v>150</v>
-      </c>
-      <c r="F55" t="s">
-        <v>150</v>
-      </c>
-      <c r="G55" t="s">
-        <v>197</v>
-      </c>
-      <c r="H55">
-        <v>0</v>
-      </c>
-      <c r="I55" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9">
-      <c r="A56" t="s">
-        <v>484</v>
-      </c>
-      <c r="B56" t="s">
-        <v>485</v>
-      </c>
-      <c r="C56" t="s">
-        <v>517</v>
-      </c>
-      <c r="D56" t="s">
-        <v>408</v>
-      </c>
-      <c r="E56" t="s">
-        <v>150</v>
-      </c>
-      <c r="F56" t="s">
-        <v>150</v>
-      </c>
-      <c r="G56" t="s">
-        <v>197</v>
-      </c>
-      <c r="H56">
-        <v>0</v>
-      </c>
-      <c r="I56" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9">
-      <c r="A57" t="s">
-        <v>486</v>
-      </c>
-      <c r="B57" t="s">
-        <v>487</v>
-      </c>
-      <c r="C57" t="s">
-        <v>517</v>
-      </c>
-      <c r="D57" t="s">
-        <v>408</v>
-      </c>
-      <c r="E57" t="s">
-        <v>150</v>
-      </c>
-      <c r="F57" t="s">
-        <v>150</v>
-      </c>
-      <c r="G57" t="s">
-        <v>197</v>
-      </c>
-      <c r="H57">
-        <v>1</v>
-      </c>
-      <c r="I57" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9">
-      <c r="A58" t="s">
-        <v>488</v>
-      </c>
-      <c r="B58" t="s">
-        <v>513</v>
-      </c>
-      <c r="C58" t="s">
-        <v>517</v>
-      </c>
-      <c r="D58" t="s">
-        <v>408</v>
-      </c>
-      <c r="E58" t="s">
-        <v>150</v>
-      </c>
-      <c r="F58" t="s">
-        <v>150</v>
-      </c>
-      <c r="G58" t="s">
-        <v>197</v>
-      </c>
-      <c r="H58">
-        <v>1</v>
-      </c>
-      <c r="I58" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9">
-      <c r="A59" t="s">
-        <v>489</v>
-      </c>
-      <c r="B59" t="s">
-        <v>512</v>
-      </c>
-      <c r="C59" t="s">
-        <v>517</v>
-      </c>
-      <c r="D59" t="s">
-        <v>490</v>
-      </c>
-      <c r="E59" t="s">
-        <v>150</v>
-      </c>
-      <c r="F59" t="s">
-        <v>150</v>
-      </c>
-      <c r="G59" t="s">
-        <v>197</v>
-      </c>
-      <c r="H59">
-        <v>1</v>
-      </c>
-      <c r="I59" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9">
-      <c r="A60" t="s">
-        <v>491</v>
-      </c>
-      <c r="B60" t="s">
-        <v>508</v>
-      </c>
-      <c r="C60" t="s">
-        <v>517</v>
-      </c>
-      <c r="D60" t="s">
-        <v>492</v>
-      </c>
-      <c r="E60" t="s">
-        <v>150</v>
-      </c>
-      <c r="F60" t="s">
-        <v>150</v>
-      </c>
-      <c r="G60" t="s">
-        <v>197</v>
-      </c>
-      <c r="H60">
-        <v>1</v>
-      </c>
-      <c r="I60" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9">
-      <c r="A61" t="s">
-        <v>493</v>
-      </c>
-      <c r="B61" t="s">
-        <v>509</v>
-      </c>
-      <c r="C61" t="s">
-        <v>517</v>
-      </c>
-      <c r="D61" t="s">
-        <v>492</v>
-      </c>
-      <c r="E61" t="s">
-        <v>150</v>
-      </c>
-      <c r="F61" t="s">
-        <v>150</v>
-      </c>
-      <c r="G61" t="s">
-        <v>197</v>
-      </c>
-      <c r="H61">
-        <v>1</v>
-      </c>
-      <c r="I61" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9">
-      <c r="A62" t="s">
-        <v>494</v>
-      </c>
-      <c r="B62" t="s">
-        <v>510</v>
-      </c>
-      <c r="C62" t="s">
-        <v>517</v>
-      </c>
-      <c r="D62" t="s">
-        <v>492</v>
-      </c>
-      <c r="E62" t="s">
-        <v>150</v>
-      </c>
-      <c r="F62" t="s">
-        <v>150</v>
-      </c>
-      <c r="G62" t="s">
-        <v>197</v>
-      </c>
-      <c r="H62">
-        <v>1</v>
-      </c>
-      <c r="I62" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9">
-      <c r="A63" t="s">
-        <v>495</v>
-      </c>
-      <c r="B63" t="s">
-        <v>496</v>
-      </c>
-      <c r="C63" t="s">
-        <v>517</v>
-      </c>
-      <c r="D63" t="s">
-        <v>497</v>
-      </c>
-      <c r="E63" t="s">
-        <v>150</v>
-      </c>
-      <c r="F63" t="s">
-        <v>150</v>
-      </c>
-      <c r="G63" t="s">
-        <v>197</v>
-      </c>
-      <c r="H63">
-        <v>0</v>
-      </c>
-      <c r="I63" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9">
-      <c r="A64" t="s">
-        <v>498</v>
-      </c>
-      <c r="B64" t="s">
-        <v>499</v>
-      </c>
-      <c r="C64" t="s">
-        <v>517</v>
-      </c>
-      <c r="D64" t="s">
-        <v>497</v>
-      </c>
-      <c r="E64" t="s">
-        <v>150</v>
-      </c>
-      <c r="F64" t="s">
-        <v>150</v>
-      </c>
-      <c r="G64" t="s">
-        <v>197</v>
-      </c>
-      <c r="H64">
-        <v>0</v>
-      </c>
-      <c r="I64" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9">
-      <c r="A65" t="s">
-        <v>500</v>
-      </c>
-      <c r="B65" t="s">
-        <v>515</v>
-      </c>
-      <c r="E65" t="s">
-        <v>150</v>
-      </c>
-      <c r="F65" t="s">
-        <v>150</v>
-      </c>
-      <c r="G65" t="s">
-        <v>197</v>
-      </c>
-      <c r="H65">
-        <v>0</v>
-      </c>
-      <c r="I65" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9">
-      <c r="A66" t="s">
-        <v>501</v>
-      </c>
-      <c r="B66" t="s">
-        <v>514</v>
-      </c>
-      <c r="E66" t="s">
-        <v>150</v>
-      </c>
-      <c r="F66" t="s">
-        <v>150</v>
-      </c>
-      <c r="G66" t="s">
-        <v>197</v>
-      </c>
-      <c r="H66">
-        <v>0</v>
-      </c>
-      <c r="I66" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9">
-      <c r="A67" t="s">
-        <v>502</v>
-      </c>
-      <c r="B67" t="s">
-        <v>516</v>
-      </c>
-      <c r="E67" t="s">
-        <v>150</v>
-      </c>
-      <c r="F67" t="s">
-        <v>150</v>
-      </c>
-      <c r="G67" t="s">
-        <v>197</v>
-      </c>
-      <c r="H67">
-        <v>0</v>
-      </c>
-      <c r="I67" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9">
-      <c r="A68" t="s">
-        <v>503</v>
-      </c>
-      <c r="B68" t="s">
-        <v>504</v>
-      </c>
-      <c r="C68" t="s">
-        <v>517</v>
-      </c>
-      <c r="D68" t="s">
-        <v>505</v>
-      </c>
-      <c r="E68" t="s">
-        <v>150</v>
-      </c>
-      <c r="F68" t="s">
-        <v>150</v>
-      </c>
-      <c r="G68" t="s">
-        <v>197</v>
-      </c>
-      <c r="H68">
-        <v>1</v>
-      </c>
-      <c r="I68" t="s">
-        <v>400</v>
+        <v>563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>